<commit_message>
Sample data: more realistic fictional dataset in the real file layouts
</commit_message>
<xml_diff>
--- a/sample/vehicle.xlsx
+++ b/sample/vehicle.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -500,6 +500,30 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>TST107</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Gray Example</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>TST108</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Harper Example</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Sample data: more realistic fictional dataset
Co-authored-by: Rimsha Shakya <rimshashakya11-dotcom@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/sample/vehicle.xlsx
+++ b/sample/vehicle.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -500,6 +500,30 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>TST107</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Gray Example</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>TST108</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Harper Example</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>